<commit_message>
add description to bird test data
</commit_message>
<xml_diff>
--- a/test_data/birds/data/additional-ro-crate-metadata.xlsx
+++ b/test_data/birds/data/additional-ro-crate-metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bbb/sandbox/ro-crate-html-lite/test_data/birds/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bbb/sandbox/casey-ro-crate-html-lite/ro-crate-html-lite/test_data/birds/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C5BA59E-5BFF-B749-9186-37DBB555C1AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B498A2E-3344-E446-B2E4-D77B3973741C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="500" windowWidth="32440" windowHeight="20500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="32440" windowHeight="18160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="80">
   <si>
     <t>name</t>
   </si>
@@ -300,7 +300,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,6 +310,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -341,7 +347,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -349,16 +355,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -760,123 +769,131 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18" style="6" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" style="6" customWidth="1"/>
-    <col min="3" max="4" width="17" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" style="3"/>
-    <col min="6" max="6" width="28.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="44" style="3" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" style="3" customWidth="1"/>
-    <col min="10" max="13" width="30" style="3" customWidth="1"/>
-    <col min="14" max="17" width="30.6640625" style="3" customWidth="1"/>
-    <col min="18" max="16384" width="8.83203125" style="3"/>
+    <col min="1" max="1" width="18" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="7" customWidth="1"/>
+    <col min="3" max="4" width="17" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17" style="5" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="2"/>
+    <col min="7" max="7" width="28.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="44" style="2" customWidth="1"/>
+    <col min="10" max="10" width="21.83203125" style="2" customWidth="1"/>
+    <col min="11" max="14" width="30" style="2" customWidth="1"/>
+    <col min="15" max="18" width="30.6640625" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:18" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>60</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="str">
+    <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="str">
         <f>LOWER(_xlfn.CONCAT("#", SUBSTITUTE(C2, " ", "_")))</f>
         <v>#magpie</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="str">
+        <f>K2</f>
+        <v>a story in language</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>75</v>
       </c>
     </row>
@@ -908,7 +925,7 @@
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B2" t="s">
@@ -919,7 +936,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B3" t="s">
@@ -930,7 +947,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B4" t="s">
@@ -941,7 +958,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B5" t="s">
@@ -1258,7 +1275,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <f>LOWER(_xlfn.CONCAT("#", SUBSTITUTE(B2, " ", "_")))</f>
         <v>#person_1</v>
       </c>

</xml_diff>